<commit_message>
updated internet issue 27,28,29
</commit_message>
<xml_diff>
--- a/12620994.xlsx
+++ b/12620994.xlsx
@@ -3218,77 +3218,144 @@
       <c r="K52" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="L52" s="18" t="s">
+      <c r="L52" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="M52" s="20" t="s">
+      <c r="M52" s="18" t="s">
         <v>53</v>
       </c>
       <c r="N52" s="19"/>
     </row>
     <row r="53">
-      <c r="A53" s="21"/>
-      <c r="B53" s="16"/>
-      <c r="C53" s="16"/>
-      <c r="D53" s="16"/>
-      <c r="E53" s="16"/>
-      <c r="F53" s="16"/>
-      <c r="G53" s="16"/>
-      <c r="H53" s="16"/>
-      <c r="I53" s="17" t="str">
+      <c r="A53" s="11">
+        <v>46292</v>
+      </c>
+      <c r="B53" s="16">
+        <v>480</v>
+      </c>
+      <c r="C53" s="16">
+        <v>0</v>
+      </c>
+      <c r="D53" s="16">
+        <v>60</v>
+      </c>
+      <c r="E53" s="16">
+        <v>35</v>
+      </c>
+      <c r="F53" s="16">
+        <v>0</v>
+      </c>
+      <c r="G53" s="16">
+        <v>0</v>
+      </c>
+      <c r="H53" s="16">
+        <v>120</v>
+      </c>
+      <c r="I53" s="17">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="17" t="str">
+        <v>695</v>
+      </c>
+      <c r="J53" s="17">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="18"/>
-      <c r="M53" s="18"/>
+        <v>745</v>
+      </c>
+      <c r="K53" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="L53" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="M53" s="18" t="s">
+        <v>53</v>
+      </c>
       <c r="N53" s="19"/>
     </row>
     <row r="54">
-      <c r="A54" s="21"/>
-      <c r="B54" s="16"/>
-      <c r="C54" s="16"/>
-      <c r="D54" s="16"/>
-      <c r="E54" s="16"/>
-      <c r="F54" s="16"/>
-      <c r="G54" s="16"/>
-      <c r="H54" s="16"/>
-      <c r="I54" s="17" t="str">
+      <c r="A54" s="11">
+        <v>46293</v>
+      </c>
+      <c r="B54" s="16">
+        <v>400</v>
+      </c>
+      <c r="C54" s="16">
+        <v>0</v>
+      </c>
+      <c r="D54" s="16">
+        <v>50</v>
+      </c>
+      <c r="E54" s="16">
+        <v>40</v>
+      </c>
+      <c r="F54" s="16">
+        <v>0</v>
+      </c>
+      <c r="G54" s="16">
+        <v>0</v>
+      </c>
+      <c r="H54" s="16">
+        <v>200</v>
+      </c>
+      <c r="I54" s="17">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="17" t="str">
+        <v>690</v>
+      </c>
+      <c r="J54" s="17">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="18"/>
-      <c r="L54" s="18"/>
-      <c r="M54" s="18"/>
+        <v>750</v>
+      </c>
+      <c r="K54" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="L54" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="M54" s="18" t="s">
+        <v>57</v>
+      </c>
       <c r="N54" s="19"/>
     </row>
     <row r="55">
-      <c r="A55" s="21"/>
-      <c r="B55" s="16"/>
-      <c r="C55" s="16"/>
-      <c r="D55" s="16"/>
-      <c r="E55" s="16"/>
-      <c r="F55" s="16"/>
-      <c r="G55" s="16"/>
-      <c r="H55" s="16"/>
-      <c r="I55" s="17" t="str">
+      <c r="A55" s="11">
+        <v>46294</v>
+      </c>
+      <c r="B55" s="16">
+        <v>500</v>
+      </c>
+      <c r="C55" s="16">
+        <v>50</v>
+      </c>
+      <c r="D55" s="16">
+        <v>70</v>
+      </c>
+      <c r="E55" s="16">
+        <v>58</v>
+      </c>
+      <c r="F55" s="16">
+        <v>0</v>
+      </c>
+      <c r="G55" s="16">
+        <v>0</v>
+      </c>
+      <c r="H55" s="16">
+        <v>150</v>
+      </c>
+      <c r="I55" s="17">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="17" t="str">
+        <v>828</v>
+      </c>
+      <c r="J55" s="17">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="18"/>
-      <c r="L55" s="18"/>
-      <c r="M55" s="18"/>
+        <v>612</v>
+      </c>
+      <c r="K55" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="L55" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="M55" s="18" t="s">
+        <v>53</v>
+      </c>
       <c r="N55" s="19"/>
     </row>
     <row r="56">
@@ -10920,7 +10987,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="lessThan" id="{A200C9DA-AB33-4994-8FA4-F7E5FD39AA8D}">
+          <x14:cfRule type="cellIs" priority="2" operator="lessThan" id="{3CFDA9BF-1AE6-4106-806C-8135A2570AA1}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -10941,7 +11008,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3" disablePrompts="0">
-        <x14:dataValidation xr:uid="{F702A3BB-8EBB-4F8C-847F-372FE0C054E2}" type="list" allowBlank="1" error="Please choose a value from the dropdown list." errorStyle="stop" imeMode="noControl" operator="between" prompt="Select today's overall feeling" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{91F4F13C-ECBA-4170-BBDF-A502D754F8D9}" type="list" allowBlank="1" error="Please choose a value from the dropdown list." errorStyle="stop" imeMode="noControl" operator="between" prompt="Select today's overall feeling" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Excellent,Good,Neutral,Low,Stressed"</xm:f>
           </x14:formula1>
@@ -10950,16 +11017,16 @@
           </x14:formula2>
           <xm:sqref>K6:K401</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{494EEC5D-975A-4FB4-8C19-ACF6A6076EFB}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="Select today's satisfaction level" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{EBC7801D-984A-4C9A-A170-5281A59ECDC2}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="Select today's satisfaction level" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Very Satisfied,Satisfied,Neutral,Unsatisfied,Very Unsatisfied"</xm:f>
           </x14:formula1>
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>L6:L51 L54:L401 L52</xm:sqref>
+          <xm:sqref>L6:L51 L56:L401 L52 L53 L54 L55</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{9A84F9B7-0B98-4554-9FF3-39EA83827984}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="Select today's energy level" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{22C882DC-E02F-49FE-984C-39D607219A87}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="Select today's energy level" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"High,Medium,Low"</xm:f>
           </x14:formula1>

</xml_diff>